<commit_message>
Switch to a low-flow adjustable pump and drop the rotameter
Replaces the 5.5 L/min fixed-speed AC pump with a brushless DC micro
pump whose speed can be turned down, so no bypass loop is needed. The
Alicat 200 sccm unit now both sets and measures the loop flow, making
the separate rotameter redundant. Tee count drops accordingly and the
pump-port fitting is marked conditional pending the new port type.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FiLuAQopRoowwbpckhcWEP
</commit_message>
<xml_diff>
--- a/docs/malzeme_listesi.xlsx
+++ b/docs/malzeme_listesi.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +43,16 @@
     <font>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00808080"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
@@ -148,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -187,11 +197,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -561,7 +575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -671,7 +685,7 @@
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>Döngüde ~21 boru ucu var. 20 yetersiz, yedekle 30.</t>
+          <t>Döngüde 21 boru ucu var. 20 yedeksiz kalıyordu, 30'a çıkarıldı.</t>
         </is>
       </c>
     </row>
@@ -709,7 +723,7 @@
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>Her sökümde yenilenir. 20'den 30'a çıkarıldı.</t>
+          <t>Her sökümde yenilenir. 20'den 30'a.</t>
         </is>
       </c>
     </row>
@@ -747,7 +761,7 @@
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>PTFE hortum için ZORUNLU. Her boru ucuna bir tane. 20'den 30'a.</t>
+          <t>PTFE hortum için ZORUNLU, her boru ucuna bir tane. 20'den 30'a.</t>
         </is>
       </c>
     </row>
@@ -790,40 +804,40 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>BAĞLANTI</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>CMC 6M-2G-S316</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Male connector, 6 mm tube x G1/8 BSPP erkek</t>
         </is>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F7" s="9" t="n"/>
-      <c r="G7" s="9">
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6">
         <f>IF(F7="","",E7*F7)</f>
         <v/>
       </c>
-      <c r="H7" s="9" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Neumo (Hy-Lok)</t>
         </is>
       </c>
-      <c r="I7" s="10" t="inlineStr">
-        <is>
-          <t>KNF pompa portları. BONDED WASHER'lı istenecek, PTFE bant işe yaramaz.</t>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>ŞARTLI: N 86'nın portu G1/8 idi. Pompa modeli değiştiği için port tipi teyit edilip bu kalem güncellenecek. Bonded washer'lı istenecek.</t>
         </is>
       </c>
     </row>
@@ -923,7 +937,7 @@
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6">
@@ -937,7 +951,7 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>1) PCD kör dalı 2) pompa bypass hattı 3) süpürme portu. 1'den 3'e.</t>
+          <t>1) PCD kör dalı 2) süpürme portu. Bypass iptal olduğu için 3'ten 2'ye indi.</t>
         </is>
       </c>
     </row>
@@ -975,7 +989,7 @@
       </c>
       <c r="I11" s="10" t="inlineStr">
         <is>
-          <t>CMC 6M-2G için yedek conta.</t>
+          <t>CMC 6M-2G için yedek conta. Port tipi değişirse bu da değişir.</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1027,7 @@
       </c>
       <c r="I12" s="13" t="inlineStr">
         <is>
-          <t>YENİ. ADM'yi partikül kirlenmesinden korur. Odacık çıkışına, PCD'den önce. Sinterlenmiş SS tercih; membran daha çok yüzey demek.</t>
+          <t>YENİ. ADM'yi partikül kirlenmesinden korur. Odacık çıkışına, PCD'den önce. Sinterlenmiş SS tercih edildi: inert ve yüzey alanı düşük.</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1047,7 @@
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>İğne vana, 6 mm sıkıştırmalı</t>
+          <t>Kapama vanası, 6 mm sıkıştırmalı</t>
         </is>
       </c>
       <c r="E13" s="11" t="n">
@@ -1051,45 +1065,45 @@
       </c>
       <c r="I13" s="13" t="inlineStr">
         <is>
-          <t>YENİ. Pompa bypass hattında, ana döngü debisini ayarlar. Mevcut iğne vana varsa alınmaz.</t>
+          <t>YENİ. Süpürme (purge) portu. Deneyler arası N2 ile hattı temizlemek için. Ölçüm sırasında kapalı.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n">
+      <c r="A14" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>BAĞLANTI</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>— (kod istenecek)</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="inlineStr">
-        <is>
-          <t>Kapama vanası, 6 mm sıkıştırmalı</t>
-        </is>
-      </c>
-      <c r="E14" s="11" t="n">
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>PTFE thread sealant (bant veya pasta)</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="12" t="n"/>
-      <c r="G14" s="12">
+      <c r="F14" s="9" t="n"/>
+      <c r="G14" s="9">
         <f>IF(F14="","",E14*F14)</f>
         <v/>
       </c>
-      <c r="H14" s="12" t="inlineStr">
-        <is>
-          <t>Neumo (Hy-Lok)</t>
-        </is>
-      </c>
-      <c r="I14" s="13" t="inlineStr">
-        <is>
-          <t>YENİ. Süpürme (purge) portu. Deneyler arası N2 ile hattı temizlemek için.</t>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>Neumo / hırdavat</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t>NPT dişleri için. İlk 1-2 diş boş bırakılır.</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1123,7 @@
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>PTFE thread sealant (bant veya pasta)</t>
+          <t>Tube cutter, 6 mm</t>
         </is>
       </c>
       <c r="E15" s="8" t="n">
@@ -1127,7 +1141,7 @@
       </c>
       <c r="I15" s="10" t="inlineStr">
         <is>
-          <t>NPT dişleri için. İlk 1-2 diş boş bırakılır.</t>
+          <t>Dik kesim şart. Falçata ferrule'ü sızdırtır.</t>
         </is>
       </c>
     </row>
@@ -1147,7 +1161,7 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>Tube cutter, 6 mm</t>
+          <t>Kaçak arama sıvısı (Snoop vb.)</t>
         </is>
       </c>
       <c r="E16" s="8" t="n">
@@ -1165,7 +1179,7 @@
       </c>
       <c r="I16" s="10" t="inlineStr">
         <is>
-          <t>Dik kesim şart. Falçata ferrule'ü sızdırtır.</t>
+          <t>Sabunlu su da olur.</t>
         </is>
       </c>
     </row>
@@ -1185,11 +1199,11 @@
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>Kaçak arama sıvısı (Snoop vb.)</t>
+          <t>Açık ağız anahtar, 14 mm ve 15 mm</t>
         </is>
       </c>
       <c r="E17" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17" s="9" t="n"/>
       <c r="G17" s="9">
@@ -1198,143 +1212,120 @@
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>Neumo / hırdavat</t>
+          <t>Hırdavat</t>
         </is>
       </c>
       <c r="I17" s="10" t="inlineStr">
         <is>
-          <t>Sabunlu su da olur.</t>
+          <t>Gövdeyi tutup somunu sıkmak için ikisi birden gerekli.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>BAĞLANTI</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>POMPA / AKIŞ</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n"/>
+      <c r="C18" s="3" t="n"/>
+      <c r="D18" s="3" t="n"/>
+      <c r="E18" s="3" t="n"/>
+      <c r="F18" s="3" t="n"/>
+      <c r="G18" s="3" t="n"/>
+      <c r="H18" s="3" t="n"/>
+      <c r="I18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>POMPA / AKIŞ</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>KNF NMP830 KTDC-B</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>Mikro diyafram pompa, 2,1 L/dk, fırçasız DC, devir ayarlı</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="12" t="n"/>
+      <c r="G19" s="12">
+        <f>IF(F19="","",E19*F19)</f>
+        <v/>
+      </c>
+      <c r="H19" s="12" t="inlineStr">
+        <is>
+          <t>KNF Türkiye</t>
+        </is>
+      </c>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>N 86 KT.18 (5,5 L/dk, 230 V AC) yerine. Fırçasız DC olduğu için devir voltaj/PWM ile düşürülür, bypass gerekmez. SİPARİŞTE BELİRT: PPS başlık + PTFE kaplı diyafram + FFKM valf (CR/EPDM olmaz). Port tipi teyit edilecek.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>POMPA / AKIŞ</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Alicat 200 sccm MFC</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>Döngü debi kontrol + ölçüm (ELİMİZDE VAR)</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="12" t="n"/>
+      <c r="G20" s="12">
+        <f>IF(F20="","",E20*F20)</f>
+        <v/>
+      </c>
+      <c r="H20" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D18" s="10" t="inlineStr">
-        <is>
-          <t>Açık ağız anahtar, 14 mm ve 15 mm</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="F18" s="9" t="n"/>
-      <c r="G18" s="9">
-        <f>IF(F18="","",E18*F18)</f>
-        <v/>
-      </c>
-      <c r="H18" s="9" t="inlineStr">
-        <is>
-          <t>Hırdavat</t>
-        </is>
-      </c>
-      <c r="I18" s="10" t="inlineStr">
-        <is>
-          <t>Gövdeyi tutup somunu sıkmak için ikisi birden gerekli.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>POMPA / AKIŞ</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
-      <c r="I19" s="4" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>POMPA / AKIŞ</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>KNF N 86 KT.18</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>Diyafram pompa, 230 V / 50 Hz, 5,5 L/dk, G1/8 port</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6">
-        <f>IF(F20="","",E20*F20)</f>
-        <v/>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>KNF Türkiye</t>
-        </is>
-      </c>
-      <c r="I20" s="7" t="inlineStr">
-        <is>
-          <t>Islak malzemeler ideal: PPS başlık + PTFE kaplı diyafram + FFPM valf. ANCAK 5,5 L/dk hedefimizin ~25 katı. Çözüm: pompa etrafına bypass (üstteki tee + iğne vana). Pompa tam devirde çalışır, ısınmaz; ana döngüye istediğimiz debi gider.</t>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>Kontrol modunda 150-200 sccm set edilir: hem debiyi belirler hem ölçer. Ayrı rotametreye gerek yok. Gaz seçimi 'Air'. Pompa çıkışı ile odacık girişi arasına.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>POMPA / AKIŞ</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>KNF NMP830 KTDC-B</t>
-        </is>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>ALTERNATİF: mikro diyafram pompa, 2,1 L/dk, fırçasız DC</t>
-        </is>
-      </c>
-      <c r="E21" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" s="12" t="n"/>
-      <c r="G21" s="12">
-        <f>IF(F21="","",E21*F21)</f>
-        <v/>
-      </c>
-      <c r="H21" s="12" t="inlineStr">
-        <is>
-          <t>KNF Türkiye</t>
-        </is>
-      </c>
-      <c r="I21" s="13" t="inlineStr">
-        <is>
-          <t>Henüz sipariş verilmediyse bunu değerlendir. Fırçasız DC olduğu için devir voltajla ayarlanır, bypass gerekmez. SORULACAK: valf malzemesi FKM veya FFKM olmalı, CR (kloropren) olmaz.</t>
-        </is>
-      </c>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>ODACIK</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n"/>
+      <c r="C21" s="3" t="n"/>
+      <c r="D21" s="3" t="n"/>
+      <c r="E21" s="3" t="n"/>
+      <c r="F21" s="3" t="n"/>
+      <c r="G21" s="3" t="n"/>
+      <c r="H21" s="3" t="n"/>
+      <c r="I21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="11" t="n">
@@ -1342,21 +1333,21 @@
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>POMPA / AKIŞ</t>
+          <t>ODACIK</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>Alicat 200 sccm MFC</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>Döngü debi ölçer (ELİMİZDE VAR)</t>
+          <t>PTFE hortum, 6 mm dış / 4 mm iç çap</t>
         </is>
       </c>
       <c r="E22" s="11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F22" s="12" t="n"/>
       <c r="G22" s="12">
@@ -1365,67 +1356,90 @@
       </c>
       <c r="H22" s="12" t="inlineStr">
         <is>
+          <t>Neumo / lab sarf</t>
+        </is>
+      </c>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>YENİ. Önceki listede insert vardı ama hortumun kendisi yoktu. Birim: metre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>ODACIK</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I22" s="13" t="inlineStr">
-        <is>
-          <t>Vana tam açık, gaz seçimi 'Air'. Hedef debi 150-200 sccm. Ayrı rotametreye gerek kalmaz.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>POMPA / AKIŞ</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>Dwyer RMA-2-SSV-VIT vb.</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>OPSİYONEL rotametre + iğne vana, 0,1-1 L/dk hava</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="n">
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>Cam kavanoz, 1 L borosilikat, geniş ağız, PTFE astarlı kapak</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F23" s="6" t="n"/>
-      <c r="G23" s="6">
+      <c r="F23" s="12" t="n"/>
+      <c r="G23" s="12">
         <f>IF(F23="","",E23*F23)</f>
         <v/>
       </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>ITM / Tetisan</t>
-        </is>
-      </c>
-      <c r="I23" s="7" t="inlineStr">
-        <is>
-          <t>DİKKAT: önceki listedeki RMA-21 modeli 1-10 L/dk. Bizim çalışma debimiz 0,15-0,5 L/dk, o skalanın en altında okunmaz. Alınacaksa düşük skalalı model alınmalı.</t>
+      <c r="H23" s="12" t="inlineStr">
+        <is>
+          <t>Lab sarf</t>
+        </is>
+      </c>
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>YENİ. Gazın biriktiği hacim burası. 30 L kutuda derişim 30 kat düşer.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>ODACIK</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n"/>
-      <c r="C24" s="3" t="n"/>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
-      <c r="F24" s="3" t="n"/>
-      <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="n"/>
-      <c r="I24" s="4" t="n"/>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>O-ring, Viton (FKM), ~11 mm iç çap x 2 mm kesit</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F24" s="9" t="n"/>
+      <c r="G24" s="9">
+        <f>IF(F24="","",E24*F24)</f>
+        <v/>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>Conta/hidrolik</t>
+        </is>
+      </c>
+      <c r="I24" s="10" t="inlineStr">
+        <is>
+          <t>Bulkhead union'ın duvara sızdırmazlığı. Karışık ölçü seti pratik.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="n">
@@ -1443,11 +1457,11 @@
       </c>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>PTFE hortum, 6 mm dış / 4 mm iç çap</t>
+          <t>Silikon conta bandı, kutu kapağı için</t>
         </is>
       </c>
       <c r="E25" s="11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F25" s="12" t="n"/>
       <c r="G25" s="12">
@@ -1456,12 +1470,12 @@
       </c>
       <c r="H25" s="12" t="inlineStr">
         <is>
-          <t>Neumo / lab sarf</t>
+          <t>Hırdavat</t>
         </is>
       </c>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>YENİ. Önceki listede insert vardı ama hortumun kendisi yoktu. Birim: metre.</t>
+          <t>YENİ. Birim: metre.</t>
         </is>
       </c>
     </row>
@@ -1476,12 +1490,12 @@
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SHT31 veya muadili</t>
         </is>
       </c>
       <c r="D26" s="13" t="inlineStr">
         <is>
-          <t>Cam kavanoz, 1 L borosilikat, geniş ağız, PTFE astarlı kapak</t>
+          <t>Sıcaklık / bağıl nem sensörü, kayıtlı</t>
         </is>
       </c>
       <c r="E26" s="11" t="n">
@@ -1494,90 +1508,67 @@
       </c>
       <c r="H26" s="12" t="inlineStr">
         <is>
+          <t>Elektronik</t>
+        </is>
+      </c>
+      <c r="I26" s="13" t="inlineStr">
+        <is>
+          <t>YENİ. Kapalı döngüde nem dengeye gelir, bunu kayıtla kanıtlamak gerekiyor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>ODACIK</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>Nitril eldiven + kelepçe (kutuya eldiven portu)</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" s="12" t="n"/>
+      <c r="G27" s="12">
+        <f>IF(F27="","",E27*F27)</f>
+        <v/>
+      </c>
+      <c r="H27" s="12" t="inlineStr">
+        <is>
           <t>Lab sarf</t>
         </is>
       </c>
-      <c r="I26" s="13" t="inlineStr">
-        <is>
-          <t>YENİ. Gazın biriktiği hacim burası. 30 L kutuda derişim 30 kat düşer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="8" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>ODACIK</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t>O-ring, Viton (FKM), ~11 mm iç çap x 2 mm kesit</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="F27" s="9" t="n"/>
-      <c r="G27" s="9">
-        <f>IF(F27="","",E27*F27)</f>
-        <v/>
-      </c>
-      <c r="H27" s="9" t="inlineStr">
-        <is>
-          <t>Conta/hidrolik</t>
-        </is>
-      </c>
-      <c r="I27" s="10" t="inlineStr">
-        <is>
-          <t>Bulkhead union'ın duvara sızdırmazlığı. Karışık ölçü seti pratik.</t>
+      <c r="I27" s="13" t="inlineStr">
+        <is>
+          <t>YENİ. Kapağı açmadan kesim yapmak için. Birim: takım.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="12" t="inlineStr">
-        <is>
-          <t>ODACIK</t>
-        </is>
-      </c>
-      <c r="C28" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
-        <is>
-          <t>Silikon conta bandı, kutu kapağı için</t>
-        </is>
-      </c>
-      <c r="E28" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" s="12" t="n"/>
-      <c r="G28" s="12">
-        <f>IF(F28="","",E28*F28)</f>
-        <v/>
-      </c>
-      <c r="H28" s="12" t="inlineStr">
-        <is>
-          <t>Hırdavat</t>
-        </is>
-      </c>
-      <c r="I28" s="13" t="inlineStr">
-        <is>
-          <t>YENİ. Birim: metre.</t>
-        </is>
-      </c>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>TEST BİLEŞİĞİ</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n"/>
+      <c r="C28" s="3" t="n"/>
+      <c r="D28" s="3" t="n"/>
+      <c r="E28" s="3" t="n"/>
+      <c r="F28" s="3" t="n"/>
+      <c r="G28" s="3" t="n"/>
+      <c r="H28" s="3" t="n"/>
+      <c r="I28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="11" t="n">
@@ -1585,17 +1576,17 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>ODACIK</t>
+          <t>TEST BİLEŞİĞİ</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>SHT31 veya muadili</t>
+          <t>CAS 119-36-8</t>
         </is>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>Sıcaklık / bağıl nem sensörü, kayıtlı</t>
+          <t>Metil salisilat, reaktif saflığı &gt;=%99, 100 mL</t>
         </is>
       </c>
       <c r="E29" s="11" t="n">
@@ -1608,12 +1599,12 @@
       </c>
       <c r="H29" s="12" t="inlineStr">
         <is>
-          <t>Elektronik</t>
+          <t>Merck / Sigma / Isolab</t>
         </is>
       </c>
       <c r="I29" s="13" t="inlineStr">
         <is>
-          <t>YENİ. Nem kaymasını kayıt altına almak için. Kapalı döngüde nem dengeye gelir ama kanıtlanmalı.</t>
+          <t>YENİ. PoC test bileşiği. Kış yeşili yağı ALINMAYACAK, o bir karışım. OSHA maruziyet sınırı yok, parlama noktası &gt;110 C, FEMA GRAS.</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1614,7 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>ODACIK</t>
+          <t>TEST BİLEŞİĞİ</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
@@ -1633,11 +1624,11 @@
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Nitril eldiven + kelepçe (kutuya eldiven portu)</t>
+          <t>Mikrolitre şırınga, 10 µL, gaz sızdırmaz</t>
         </is>
       </c>
       <c r="E30" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30" s="12" t="n"/>
       <c r="G30" s="12">
@@ -1651,223 +1642,163 @@
       </c>
       <c r="I30" s="13" t="inlineStr">
         <is>
-          <t>YENİ. Kapağı açmadan kesim yapmak için. Birim: takım.</t>
+          <t>YENİ. Tek doz 0,2-1 µL. 1 L kavanozda 0,2 µL yaklaşık 27 ppm eder.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>TEST BİLEŞİĞİ</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="n"/>
-      <c r="C31" s="3" t="n"/>
-      <c r="D31" s="3" t="n"/>
-      <c r="E31" s="3" t="n"/>
-      <c r="F31" s="3" t="n"/>
-      <c r="G31" s="3" t="n"/>
-      <c r="H31" s="3" t="n"/>
-      <c r="I31" s="4" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="11" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="12" t="inlineStr">
-        <is>
-          <t>TEST BİLEŞİĞİ</t>
-        </is>
-      </c>
-      <c r="C32" s="12" t="inlineStr">
-        <is>
-          <t>CAS 119-36-8</t>
-        </is>
-      </c>
-      <c r="D32" s="13" t="inlineStr">
-        <is>
-          <t>Metil salisilat, reaktif saflığı &gt;=%99, 100 mL</t>
-        </is>
-      </c>
-      <c r="E32" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" s="12" t="n"/>
-      <c r="G32" s="12">
-        <f>IF(F32="","",E32*F32)</f>
-        <v/>
-      </c>
-      <c r="H32" s="12" t="inlineStr">
-        <is>
-          <t>Merck / Sigma / Isolab</t>
-        </is>
-      </c>
-      <c r="I32" s="13" t="inlineStr">
-        <is>
-          <t>YENİ. PoC test bileşiği. Kış yeşili yağı ALINMAYACAK, o bir karışım. OSHA maruziyet sınırı yok, parlama noktası &gt;110 C, FEMA GRAS.</t>
-        </is>
-      </c>
+      <c r="A31" s="14" t="n"/>
+      <c r="B31" s="14" t="n"/>
+      <c r="C31" s="14" t="n"/>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>TOPLAM</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="n"/>
+      <c r="F31" s="14" t="n"/>
+      <c r="G31" s="15">
+        <f>SUM(G2:G30)</f>
+        <v/>
+      </c>
+      <c r="H31" s="14" t="n"/>
+      <c r="I31" s="14" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>TEST BİLEŞİĞİ</t>
-        </is>
-      </c>
-      <c r="C33" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
-        <is>
-          <t>Mikrolitre şırınga, 10 µL, gaz sızdırmaz</t>
-        </is>
-      </c>
-      <c r="E33" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F33" s="12" t="n"/>
-      <c r="G33" s="12">
-        <f>IF(F33="","",E33*F33)</f>
-        <v/>
-      </c>
-      <c r="H33" s="12" t="inlineStr">
-        <is>
-          <t>Lab sarf</t>
-        </is>
-      </c>
-      <c r="I33" s="13" t="inlineStr">
-        <is>
-          <t>YENİ. Tek doz 0,2-1 µL. 1 L kavanozda 0,2 µL ~ 27 ppm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="14" t="n"/>
-      <c r="B34" s="14" t="n"/>
-      <c r="C34" s="14" t="n"/>
-      <c r="D34" s="15" t="inlineStr">
-        <is>
-          <t>TOPLAM</t>
-        </is>
-      </c>
-      <c r="E34" s="14" t="n"/>
-      <c r="F34" s="14" t="n"/>
-      <c r="G34" s="15">
-        <f>SUM(G2:G33)</f>
-        <v/>
-      </c>
-      <c r="H34" s="14" t="n"/>
-      <c r="I34" s="14" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="16" t="inlineStr">
-        <is>
-          <t>LEJANT</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="17" t="inlineStr">
-        <is>
-          <t>Sarı = yeni eklendi</t>
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>İPTAL EDİLENLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>KNF N 86 KT.18 (5,5 L/dk, 230 V AC) - debisi hedefin 25 katı ve sabit devir. Yerine NMP830 KTDC-B.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="15" customHeight="1">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>Dwyer RMA-21-SSV-VIT rotametre (1-10 L/dk) - hem skalası yanlıştı hem de MFC entegre edildiği için gereksiz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="15" customHeight="1">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>Pompa bypass hattı (tee + iğne vana) - pompa debisi doğrudan düşürüleceği için gerekmiyor.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="18" t="inlineStr">
         <is>
-          <t>Turuncu = adet veya model değiştirildi</t>
+          <t>LEJANT</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="19" t="inlineStr">
         <is>
+          <t>Sarı = yeni eklendi</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="20" t="inlineStr">
+        <is>
+          <t>Turuncu = adet veya model değiştirildi</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="21" t="inlineStr">
+        <is>
           <t>Renksiz = önceki listeden aynen geldi</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="20" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="22" t="inlineStr">
         <is>
           <t>SİPARİŞ ÖNCESİ DOĞRULANACAKLAR</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="26" customHeight="1">
-      <c r="A42" s="21" t="inlineStr">
-        <is>
-          <t>1. ADM01'in gaz portu ölçüsü. Thorlabs ADM01 Hy-Lok rakorla geliyor ama 1/4" mi 6 mm mi fiziksel olarak ölçülmeli. Mevcut hatta zaten bağlı olduğu için oradaki rakorlar tekrar kullanılabilir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="26" customHeight="1">
-      <c r="A43" s="21" t="inlineStr">
-        <is>
-          <t>2. Alicat MFC ve PCD port tipleri. Liste 1/8" NPT varsayıyor (PCD'de takılı olan '9A' damgalı connector bunu doğruluyor). MFC için cihazın üstünden teyit edilmeli.</t>
-        </is>
-      </c>
-    </row>
     <row r="44" ht="26" customHeight="1">
-      <c r="A44" s="21" t="inlineStr">
-        <is>
-          <t>3. Hy-Lok gövdeleri (tee, bulkhead, connector) somun+ferrule takılı mı geliyor? Genelde evet. Neumo'ya sorulmalı, yoksa somun/ferrule adedi artırılmalı.</t>
+      <c r="A44" s="23" t="inlineStr">
+        <is>
+          <t>1. ADM01'in gaz portu ölçüsü. Thorlabs ADM01 Hy-Lok rakorla geliyor ama 1/4" mi 6 mm mi katalogda yazmıyor. Mevcut hatta zaten bağlı, oradaki rakor ölçülerek teyit edilecek.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="26" customHeight="1">
-      <c r="A45" s="21" t="inlineStr">
-        <is>
-          <t>4. KNF NMP830 KTDC valf malzemesi. FKM veya FFKM olmalı; CR (kloropren) uçucuları emer.</t>
+      <c r="A45" s="23" t="inlineStr">
+        <is>
+          <t>2. NMP830'un port tipi (G1/8 diş mi, hortum nipeli mi). CMC 6M-2G kalemi buna göre güncellenecek.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="26" customHeight="1">
-      <c r="A46" s="21" t="inlineStr">
-        <is>
-          <t>5. Filtre ve vana kodları Neumo'dan istenecek. 6 mm sıkıştırmalı uçlu, 2 µm eleman.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="22" t="inlineStr">
+      <c r="A46" s="23" t="inlineStr">
+        <is>
+          <t>3. Alicat MFC ve PCD port tipleri. Liste 1/8" NPT varsayıyor; PCD'de takılı '9A' damgalı connector bunu doğruluyor, MFC cihazın üstünden teyit edilecek.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="26" customHeight="1">
+      <c r="A47" s="23" t="inlineStr">
+        <is>
+          <t>4. Hy-Lok gövdeleri (tee, bulkhead, connector) somun+ferrule takılı mı geliyor? Genelde evet; değilse somun/ferrule adedi artırılacak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="26" customHeight="1">
+      <c r="A48" s="23" t="inlineStr">
+        <is>
+          <t>5. Filtre ve kapama vanası kodları Neumo'dan istenecek: 6 mm sıkıştırmalı uçlu, filtre elemanı 2 µm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="24" t="inlineStr">
         <is>
           <t>DÖNGÜ SIRASI</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="19" t="inlineStr">
-        <is>
-          <t>Odacık çıkışı -&gt; Filtre -&gt; PCD (T ile kör dal) -&gt; ADM -&gt; Pompa -&gt; İğne vana (bypass) -&gt; MFC -&gt; Odacık girişi</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="26" customHeight="1">
-      <c r="A50" s="21" t="inlineStr">
-        <is>
-          <t>Kısma her zaman pompadan SONRA. Böylece ADM emme tarafında, odacık basıncında kalır; pompa çıkışı ile vana arası dışında hiçbir yerde basınç yükselmez.</t>
+    <row r="51" ht="26" customHeight="1">
+      <c r="A51" s="23" t="inlineStr">
+        <is>
+          <t>Odacık çıkışı -&gt; Filtre -&gt; PCD (T ile kör dal) -&gt; ADM -&gt; Pompa -&gt; MFC -&gt; Odacık girişi</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="26" customHeight="1">
+      <c r="A52" s="23" t="inlineStr">
+        <is>
+          <t>Debiyi pompanın devri kabaca, MFC ince olarak belirler. ADM pompanın emme tarafında kaldığı için odacık basıncında çalışır; hiçbir yerde basınç yükselmez. Hedef debi 150-200 sccm, 1 L kavanozu 5-7 dakikada çevirir.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A43:I43"/>
-    <mergeCell ref="A19:I19"/>
+  <mergeCells count="14">
+    <mergeCell ref="A52:I52"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A49:I49"/>
-    <mergeCell ref="A42:I42"/>
+    <mergeCell ref="A51:I51"/>
+    <mergeCell ref="A47:I47"/>
+    <mergeCell ref="A28:I28"/>
     <mergeCell ref="A46:I46"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A44:I44"/>
     <mergeCell ref="A45:I45"/>
-    <mergeCell ref="A31:I31"/>
-    <mergeCell ref="A50:I50"/>
-    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A34:I34"/>
+    <mergeCell ref="A35:I35"/>
+    <mergeCell ref="A48:I48"/>
+    <mergeCell ref="A21:I21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>

</xml_diff>

<commit_message>
Spec the pump by required flow instead of a fixed model
2.1 L/min is 2100 sccm, about ten times the 150-300 sccm the loop needs,
so the pump line now carries the requirement (flow band, PTFE-coated
diaphragm, FFKM valves, brushless DC) for the supplier to match, with the
candidate series and their trade-offs in the note. Also drops the fitting
verification item: the 6 mm sizing is already confirmed by the existing
gas line and the earlier order.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FiLuAQopRoowwbpckhcWEP
</commit_message>
<xml_diff>
--- a/docs/malzeme_listesi.xlsx
+++ b/docs/malzeme_listesi.xlsx
@@ -158,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -210,6 +210,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1236,41 +1242,41 @@
       <c r="H18" s="3" t="n"/>
       <c r="I18" s="4" t="n"/>
     </row>
-    <row r="19">
-      <c r="A19" s="11" t="n">
+    <row r="19" ht="58" customHeight="1">
+      <c r="A19" s="25" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B19" s="26" t="inlineStr">
         <is>
           <t>POMPA / AKIŞ</t>
         </is>
       </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>KNF NMP830 KTDC-B</t>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>KNF — model istenecek</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>Mikro diyafram pompa, 2,1 L/dk, fırçasız DC, devir ayarlı</t>
-        </is>
-      </c>
-      <c r="E19" s="11" t="n">
+          <t>Mikro diyafram pompa, çalışma debisi 150–300 sccm, fırçasız DC</t>
+        </is>
+      </c>
+      <c r="E19" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="12" t="n"/>
-      <c r="G19" s="12">
+      <c r="F19" s="26" t="n"/>
+      <c r="G19" s="26">
         <f>IF(F19="","",E19*F19)</f>
         <v/>
       </c>
-      <c r="H19" s="12" t="inlineStr">
+      <c r="H19" s="26" t="inlineStr">
         <is>
           <t>KNF Türkiye</t>
         </is>
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>N 86 KT.18 (5,5 L/dk, 230 V AC) yerine. Fırçasız DC olduğu için devir voltaj/PWM ile düşürülür, bypass gerekmez. SİPARİŞTE BELİRT: PPS başlık + PTFE kaplı diyafram + FFKM valf (CR/EPDM olmaz). Port tipi teyit edilecek.</t>
+          <t>ŞARTNAME KNF TÜRKİYE'YE VERİLECEK: 150–300 sccm çalışma debisi, PPS/PTFE ıslak yüzey, PTFE kaplı diyafram, FFKM valf, fırçasız DC (devir ayarlı). NMP 03 / NMP 05 serisi debi olarak uygun ama PTFE diyafram 'talep üzerine' — teyit edilecek. NMP830 KTDC-B'de PTFE+FFKM standart ama debisi 2100 sccm, yani hedefin 10 katı; son çare olarak devri kısılıp MFC ile kontrol edilerek kullanılabilir.</t>
         </is>
       </c>
     </row>
@@ -1664,6 +1670,7 @@
       <c r="H31" s="14" t="n"/>
       <c r="I31" s="14" t="n"/>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
         <is>
@@ -1692,6 +1699,7 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="18" t="inlineStr">
         <is>
@@ -1720,6 +1728,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="22" t="inlineStr">
         <is>
@@ -1730,14 +1739,14 @@
     <row r="44" ht="26" customHeight="1">
       <c r="A44" s="23" t="inlineStr">
         <is>
-          <t>1. ADM01'in gaz portu ölçüsü. Thorlabs ADM01 Hy-Lok rakorla geliyor ama 1/4" mi 6 mm mi katalogda yazmıyor. Mevcut hatta zaten bağlı, oradaki rakor ölçülerek teyit edilecek.</t>
+          <t>1. Rakor ölçüleri (6 mm) önceki siparişten teyitli — ADM01, PCD ve MFC hattı zaten bu ölçüde kurulu. PCD'de takılı '9A' damgalı connector 1/8" NPT'yi doğruluyor. Yeni doğrulama gerekmiyor.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="26" customHeight="1">
       <c r="A45" s="23" t="inlineStr">
         <is>
-          <t>2. NMP830'un port tipi (G1/8 diş mi, hortum nipeli mi). CMC 6M-2G kalemi buna göre güncellenecek.</t>
+          <t>2. Seçilecek pompanın port tipi (G1/8 diş mi, hortum nipeli mi). CMC 6M-2G kalemi buna göre güncellenecek.</t>
         </is>
       </c>
     </row>
@@ -1762,6 +1771,7 @@
         </is>
       </c>
     </row>
+    <row r="49"/>
     <row r="50">
       <c r="A50" s="24" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Open the pump line to other brands and flag the insert lead time
Drops the single-vendor assumption: the PTFE-diaphragm requirement is
what forces oversized units, so the spec now asks for FKM or better at
the right flow and lists candidate suppliers, including the Parker micro
pump the reference plant-VOC paper used at 480 sccm. Also records the
four-to-five week lead time on the tube inserts from the January quote.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FiLuAQopRoowwbpckhcWEP
</commit_message>
<xml_diff>
--- a/docs/malzeme_listesi.xlsx
+++ b/docs/malzeme_listesi.xlsx
@@ -158,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -210,6 +210,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -733,7 +739,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="5" t="n">
         <v>4</v>
       </c>
@@ -767,7 +773,7 @@
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>PTFE hortum için ZORUNLU, her boru ucuna bir tane. 20'den 30'a.</t>
+          <t>PTFE hortum için ZORUNLU, her boru ucuna bir tane. 20'den 30'a. DİKKAT: 23.01.2026 teklifinde teslim süresi 4-5 HAFTA (somun ve ferrule stokta). Sipariş sırasında bu kalemi öne al. Birim fiyat ~1,42 EUR.</t>
         </is>
       </c>
     </row>
@@ -1000,15 +1006,15 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n">
+      <c r="A12" s="25" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>BAĞLANTI</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C12" s="26" t="inlineStr">
         <is>
           <t>— (kod istenecek)</t>
         </is>
@@ -1018,15 +1024,15 @@
           <t>Hat içi filtre, 6 mm sıkıştırmalı, 2 µm sinterlenmiş SS eleman</t>
         </is>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="12" t="n"/>
-      <c r="G12" s="12">
+      <c r="F12" s="26" t="n"/>
+      <c r="G12" s="26">
         <f>IF(F12="","",E12*F12)</f>
         <v/>
       </c>
-      <c r="H12" s="12" t="inlineStr">
+      <c r="H12" s="26" t="inlineStr">
         <is>
           <t>Neumo (Hy-Lok)</t>
         </is>
@@ -1038,15 +1044,15 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n">
+      <c r="A13" s="25" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="26" t="inlineStr">
         <is>
           <t>BAĞLANTI</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C13" s="26" t="inlineStr">
         <is>
           <t>— (kod istenecek)</t>
         </is>
@@ -1056,15 +1062,15 @@
           <t>Kapama vanası, 6 mm sıkıştırmalı</t>
         </is>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="12" t="n"/>
-      <c r="G13" s="12">
+      <c r="F13" s="26" t="n"/>
+      <c r="G13" s="26">
         <f>IF(F13="","",E13*F13)</f>
         <v/>
       </c>
-      <c r="H13" s="12" t="inlineStr">
+      <c r="H13" s="26" t="inlineStr">
         <is>
           <t>Neumo (Hy-Lok)</t>
         </is>
@@ -1242,18 +1248,18 @@
       <c r="H18" s="3" t="n"/>
       <c r="I18" s="4" t="n"/>
     </row>
-    <row r="19" ht="58" customHeight="1">
-      <c r="A19" s="25" t="n">
+    <row r="19" ht="86" customHeight="1">
+      <c r="A19" s="27" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="26" t="inlineStr">
+      <c r="B19" s="28" t="inlineStr">
         <is>
           <t>POMPA / AKIŞ</t>
         </is>
       </c>
-      <c r="C19" s="26" t="inlineStr">
-        <is>
-          <t>KNF — model istenecek</t>
+      <c r="C19" s="28" t="inlineStr">
+        <is>
+          <t>Marka serbest — model istenecek</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
@@ -1261,35 +1267,35 @@
           <t>Mikro diyafram pompa, çalışma debisi 150–300 sccm, fırçasız DC</t>
         </is>
       </c>
-      <c r="E19" s="25" t="n">
+      <c r="E19" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="26" t="n"/>
-      <c r="G19" s="26">
+      <c r="F19" s="28" t="n"/>
+      <c r="G19" s="28">
         <f>IF(F19="","",E19*F19)</f>
         <v/>
       </c>
-      <c r="H19" s="26" t="inlineStr">
-        <is>
-          <t>KNF Türkiye</t>
+      <c r="H19" s="28" t="inlineStr">
+        <is>
+          <t>Parker / Schwarzer / Thomas / KNF — teklif alınacak</t>
         </is>
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>ŞARTNAME KNF TÜRKİYE'YE VERİLECEK: 150–300 sccm çalışma debisi, PPS/PTFE ıslak yüzey, PTFE kaplı diyafram, FFKM valf, fırçasız DC (devir ayarlı). NMP 03 / NMP 05 serisi debi olarak uygun ama PTFE diyafram 'talep üzerine' — teyit edilecek. NMP830 KTDC-B'de PTFE+FFKM standart ama debisi 2100 sccm, yani hedefin 10 katı; son çare olarak devri kısılıp MFC ile kontrol edilerek kullanılabilir.</t>
+          <t>ŞARTNAME: 150–300 sccm çalışma debisi, sızdırmaz (kapalı döngü), fırçasız DC (devir ayarlı), ıslak malzeme FKM (Viton) veya daha iyisi — NBR ve EPDM OLMAZ, organikleri emip geri salar. PTFE kaplı diyafram ideal ama şart değil; PTFE ısrarı bizi 2000 sccm'lik pompalara zorluyor, debi uyumu malzemeden daha önemli çünkü ölçümümüz kesim öncesi/sonrası farkı. ADAYLAR: Parker Hannifin T5/T2 serisi (Li 2019 bitki VOC örneklemesinde T5-1IC-03-1EEP'i 480 sccm'de kullanmış — literatür örneği var), Schwarzer Precision SP serisi, Thomas / Gardner Denver, Xavitech V serisi (devir kontrolü dahili), Boxer, TCS Micropumps. KNF de teklif versin ama tek seçenek değil. ELEME: Air Dimensions Dia-Vac — malzemesi ideal ama en küçüğü 13 L/dk, çok büyük.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="n">
+      <c r="A20" s="25" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="26" t="inlineStr">
         <is>
           <t>POMPA / AKIŞ</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr">
+      <c r="C20" s="26" t="inlineStr">
         <is>
           <t>Alicat 200 sccm MFC</t>
         </is>
@@ -1299,15 +1305,15 @@
           <t>Döngü debi kontrol + ölçüm (ELİMİZDE VAR)</t>
         </is>
       </c>
-      <c r="E20" s="11" t="n">
+      <c r="E20" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="F20" s="12" t="n"/>
-      <c r="G20" s="12">
+      <c r="F20" s="26" t="n"/>
+      <c r="G20" s="26">
         <f>IF(F20="","",E20*F20)</f>
         <v/>
       </c>
-      <c r="H20" s="12" t="inlineStr">
+      <c r="H20" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1334,15 +1340,15 @@
       <c r="I21" s="4" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="n">
+      <c r="A22" s="25" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B22" s="26" t="inlineStr">
         <is>
           <t>ODACIK</t>
         </is>
       </c>
-      <c r="C22" s="12" t="inlineStr">
+      <c r="C22" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1352,15 +1358,15 @@
           <t>PTFE hortum, 6 mm dış / 4 mm iç çap</t>
         </is>
       </c>
-      <c r="E22" s="11" t="n">
+      <c r="E22" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="F22" s="12" t="n"/>
-      <c r="G22" s="12">
+      <c r="F22" s="26" t="n"/>
+      <c r="G22" s="26">
         <f>IF(F22="","",E22*F22)</f>
         <v/>
       </c>
-      <c r="H22" s="12" t="inlineStr">
+      <c r="H22" s="26" t="inlineStr">
         <is>
           <t>Neumo / lab sarf</t>
         </is>
@@ -1372,15 +1378,15 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="n">
+      <c r="A23" s="25" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B23" s="26" t="inlineStr">
         <is>
           <t>ODACIK</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr">
+      <c r="C23" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1390,15 +1396,15 @@
           <t>Cam kavanoz, 1 L borosilikat, geniş ağız, PTFE astarlı kapak</t>
         </is>
       </c>
-      <c r="E23" s="11" t="n">
+      <c r="E23" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="F23" s="12" t="n"/>
-      <c r="G23" s="12">
+      <c r="F23" s="26" t="n"/>
+      <c r="G23" s="26">
         <f>IF(F23="","",E23*F23)</f>
         <v/>
       </c>
-      <c r="H23" s="12" t="inlineStr">
+      <c r="H23" s="26" t="inlineStr">
         <is>
           <t>Lab sarf</t>
         </is>
@@ -1448,15 +1454,15 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="n">
+      <c r="A25" s="25" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B25" s="26" t="inlineStr">
         <is>
           <t>ODACIK</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr">
+      <c r="C25" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1466,15 +1472,15 @@
           <t>Silikon conta bandı, kutu kapağı için</t>
         </is>
       </c>
-      <c r="E25" s="11" t="n">
+      <c r="E25" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="F25" s="12" t="n"/>
-      <c r="G25" s="12">
+      <c r="F25" s="26" t="n"/>
+      <c r="G25" s="26">
         <f>IF(F25="","",E25*F25)</f>
         <v/>
       </c>
-      <c r="H25" s="12" t="inlineStr">
+      <c r="H25" s="26" t="inlineStr">
         <is>
           <t>Hırdavat</t>
         </is>
@@ -1486,15 +1492,15 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="n">
+      <c r="A26" s="25" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B26" s="26" t="inlineStr">
         <is>
           <t>ODACIK</t>
         </is>
       </c>
-      <c r="C26" s="12" t="inlineStr">
+      <c r="C26" s="26" t="inlineStr">
         <is>
           <t>SHT31 veya muadili</t>
         </is>
@@ -1504,15 +1510,15 @@
           <t>Sıcaklık / bağıl nem sensörü, kayıtlı</t>
         </is>
       </c>
-      <c r="E26" s="11" t="n">
+      <c r="E26" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="F26" s="12" t="n"/>
-      <c r="G26" s="12">
+      <c r="F26" s="26" t="n"/>
+      <c r="G26" s="26">
         <f>IF(F26="","",E26*F26)</f>
         <v/>
       </c>
-      <c r="H26" s="12" t="inlineStr">
+      <c r="H26" s="26" t="inlineStr">
         <is>
           <t>Elektronik</t>
         </is>
@@ -1524,15 +1530,15 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="n">
+      <c r="A27" s="25" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B27" s="26" t="inlineStr">
         <is>
           <t>ODACIK</t>
         </is>
       </c>
-      <c r="C27" s="12" t="inlineStr">
+      <c r="C27" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1542,15 +1548,15 @@
           <t>Nitril eldiven + kelepçe (kutuya eldiven portu)</t>
         </is>
       </c>
-      <c r="E27" s="11" t="n">
+      <c r="E27" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="F27" s="12" t="n"/>
-      <c r="G27" s="12">
+      <c r="F27" s="26" t="n"/>
+      <c r="G27" s="26">
         <f>IF(F27="","",E27*F27)</f>
         <v/>
       </c>
-      <c r="H27" s="12" t="inlineStr">
+      <c r="H27" s="26" t="inlineStr">
         <is>
           <t>Lab sarf</t>
         </is>
@@ -1577,15 +1583,15 @@
       <c r="I28" s="4" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="n">
+      <c r="A29" s="25" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="26" t="inlineStr">
         <is>
           <t>TEST BİLEŞİĞİ</t>
         </is>
       </c>
-      <c r="C29" s="12" t="inlineStr">
+      <c r="C29" s="26" t="inlineStr">
         <is>
           <t>CAS 119-36-8</t>
         </is>
@@ -1595,15 +1601,15 @@
           <t>Metil salisilat, reaktif saflığı &gt;=%99, 100 mL</t>
         </is>
       </c>
-      <c r="E29" s="11" t="n">
+      <c r="E29" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="F29" s="12" t="n"/>
-      <c r="G29" s="12">
+      <c r="F29" s="26" t="n"/>
+      <c r="G29" s="26">
         <f>IF(F29="","",E29*F29)</f>
         <v/>
       </c>
-      <c r="H29" s="12" t="inlineStr">
+      <c r="H29" s="26" t="inlineStr">
         <is>
           <t>Merck / Sigma / Isolab</t>
         </is>
@@ -1615,15 +1621,15 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="n">
+      <c r="A30" s="25" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B30" s="26" t="inlineStr">
         <is>
           <t>TEST BİLEŞİĞİ</t>
         </is>
       </c>
-      <c r="C30" s="12" t="inlineStr">
+      <c r="C30" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1633,15 +1639,15 @@
           <t>Mikrolitre şırınga, 10 µL, gaz sızdırmaz</t>
         </is>
       </c>
-      <c r="E30" s="11" t="n">
+      <c r="E30" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="F30" s="12" t="n"/>
-      <c r="G30" s="12">
+      <c r="F30" s="26" t="n"/>
+      <c r="G30" s="26">
         <f>IF(F30="","",E30*F30)</f>
         <v/>
       </c>
-      <c r="H30" s="12" t="inlineStr">
+      <c r="H30" s="26" t="inlineStr">
         <is>
           <t>Lab sarf</t>
         </is>

</xml_diff>